<commit_message>
Correct Mode 5 QA doc: FG delivery COGS finding was a false alarm, not a bug
TC-E2E-M5-12 originally flagged "FG delivery posts no COGS" as an unfixed
bug. Deeper investigation (tracing Odoo core's _run_fifo in stock_account)
found the real cause: this product had 5 pre-existing units in stock
valued at ฿0 (a known, already-accepted historical gap from before
ADR-049's labor-cost fix). The two fixture deliveries happened to consume
exactly those 5 zero-cost units before touching the freshly-produced,
correctly-valued batch — FIFO working exactly as designed, not a defect.
Added a third real SO/delivery/invoice (S00114, fresh stock only) proving
the mechanism posts COGS correctly (dr 511100 COGS / cr 113150 Inventory,
฿933.33 exact). No code change needed. Updated doc, banner, and library
card to reflect the corrected finding.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode5.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode5.xlsx
@@ -1552,12 +1552,12 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>ตรวจรายการบัญชีของใบแจ้งหนี้ (Journal Items)</t>
+          <t>ตรวจรายการบัญชีของใบแจ้งหนี้ (Journal Items) — ยืนยันว่าลง COGS ถูกต้อง</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-11 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M5-11 เสร็จแล้ว (ตัวอย่างนี้ใช้ SO/Invoice อีกใบที่ขายจาก FG ล็อตใหม่ล้วน เพื่อให้เห็นรายการ COGS จริง)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>เดบิต/เครดิตสมดุลกัน (รวมเท่ากันทั้ง 2 ฝั่ง) — ตัวอย่างจริง: INV/2026/00018 เดบิต Trade Receivables 48,150.00 บาท = เครดิต Sales Revenue - FG Production 45,000.00 + Output VAT 3,150.00 บาท (ไม่มีรายการ COGS ปรากฏเลย — ดูหมายเหตุสีแดงด้านบน)</t>
+          <t>เดบิต/เครดิตสมดุลกัน (รวมเท่ากันทั้ง 2 ฝั่ง) พร้อมมีรายการ COGS ปรากฏครบ — ตัวอย่างจริง: INV/2026/00020 (SO S00114, ขาย FG ล็อตใหม่ 2 หน่วย) เดบิต Trade Receivables 32,100.00 = เครดิต Sales Revenue - FG Production 30,000.00 + Output VAT 2,100.00 บาท และมีคู่ COGS แยกสมดุลกันเอง: เดบิต 511100 Cost of Goods Sold 933.33 = เครดิต 113150 Inventory - Stone FG 933.33 บาท (933.33 = 466.67 บาท/หน่วย × 2 หน่วย ตรงกับต้นทุน Slab จริงเป๊ะ)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>🔴 พบปัญหาจริง (ยังไม่ได้แก้ไข แจ้งผู้ใช้แล้ว): ใบส่งของ (Delivery) ของ FG ไม่ได้ลงบัญชีต้นทุนขาย (COGS) เลยสักบาท — มูลค่า Slab ที่ใช้ผลิต (2,800.00 บาท) ที่โอนเข้าบัญชี "Inventory - Stone FG" ตอนผลิตเสร็จ ค้างอยู่ในบัญชีนั้นตลอดไป ต่อให้สินค้าถูกส่งมอบให้ลูกค้าไปแล้วก็ตาม — ต่างจาก Mode 1/2/3 ที่มีการโอนต้นทุนออกตอนส่งของ/ออกใบแจ้งหนี้ให้เห็นชัดเจน</t>
+          <t>ℹ️ หมายเหตุ: ใบแจ้งหนี้ของ S00112/S00113 เองไม่มีรายการ COGS ขึ้นมา — ตอนแรกเข้าใจผิดว่าเป็นบั๊ก แต่ตรวจสอบลึกแล้วพบว่าไม่ใช่: หินที่ส่งมอบ 5 หน่วยในนั้นตรงกับสต็อกเก่าที่มีอยู่แล้ว 5 หน่วยพอดี ซึ่งเป็นข้อมูลสาธิตเก่าที่มีมูลค่าบันทึกไว้ 0.00 บาทตั้งแต่ต้น (ช่องว่างข้อมูลที่รู้และยอมรับไว้แล้วก่อนหน้านี้ ไม่ใช่ปัญหาใหม่) ระบบคิดต้นทุนแบบ FIFO จึงตัดจากของเก่า (มูลค่า 0) ก่อนของใหม่ที่เพิ่งผลิตถูกต้องแล้วตามหลัก FIFO — ไม่ใช่บั๊กของ Mode 5 เลย ดูตัวอย่างที่ยืนยันว่าระบบลงบัญชีถูกต้องจริงด้านล่าง (ใช้ของใหม่ล้วน ไม่ปนของเก่า)</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>

</xml_diff>